<commit_message>
test: restore malformed shared string references
</commit_message>
<xml_diff>
--- a/tests/fixtures/invalid_shared_strings.xlsx
+++ b/tests/fixtures/invalid_shared_strings.xlsx
@@ -1576,7 +1576,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
   <dimension ref="A1:C105"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="14.25" outlineLevelCol="2"/>
@@ -1589,15 +1589,15 @@
     <row r="1" ht="42" customHeight="1"/>
     <row r="3" ht="22" customHeight="1" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>0</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1</v>
+        <v>257</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2">

</xml_diff>